<commit_message>
minor changes (and T3 for lab1 matlogic added)
</commit_message>
<xml_diff>
--- a/_Studying(5th_sem)/ElectricalAndSchemotechnicalEngineering/лаб3/Лист Microsoft Excel.xlsx
+++ b/_Studying(5th_sem)/ElectricalAndSchemotechnicalEngineering/лаб3/Лист Microsoft Excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\itmo\_Studying(5th_sem)\ElectricalAndSchemotechnicalEngineering\лаб3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86B5F358-12A2-45A4-9A47-31A41558DAFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E1DB4E3-4D43-40CC-A459-3E065CEEFE1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="24892" windowHeight="14914" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -429,16 +429,16 @@
         <v>0.5</v>
       </c>
       <c r="B2">
+        <v>2.351</v>
+      </c>
+      <c r="C2">
         <v>1.2490000000000001</v>
       </c>
-      <c r="C2">
-        <v>2.351</v>
-      </c>
       <c r="D2">
+        <v>0.67900000000000005</v>
+      </c>
+      <c r="E2">
         <v>0.64800000000000002</v>
-      </c>
-      <c r="E2">
-        <v>0.67900000000000005</v>
       </c>
       <c r="F2">
         <f>AVERAGE(B2:C2)</f>
@@ -447,29 +447,37 @@
       <c r="G2">
         <v>2.1800000000000002</v>
       </c>
+      <c r="H2">
+        <f>G2/(2*A2)</f>
+        <v>2.1800000000000002</v>
+      </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A3">
         <v>0.75</v>
       </c>
       <c r="B3">
+        <v>2.367</v>
+      </c>
+      <c r="C3">
         <v>1.08</v>
       </c>
-      <c r="C3">
-        <v>2.367</v>
-      </c>
       <c r="D3">
+        <v>0.68100000000000005</v>
+      </c>
+      <c r="E3">
         <v>0.61699999999999999</v>
       </c>
-      <c r="E3">
-        <v>0.68100000000000005</v>
-      </c>
       <c r="F3">
-        <f t="shared" ref="F3:F4" si="0">AVERAGE(B3:C3)</f>
+        <f>AVERAGE(B3:C3)</f>
         <v>1.7235</v>
       </c>
       <c r="G3">
         <v>3.25</v>
+      </c>
+      <c r="H3">
+        <f t="shared" ref="H3:H4" si="0">G3/(2*A3)</f>
+        <v>2.1666666666666665</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.4">
@@ -477,23 +485,27 @@
         <v>1</v>
       </c>
       <c r="B4">
+        <v>2.1269999999999998</v>
+      </c>
+      <c r="C4">
         <v>1.0269999999999999</v>
       </c>
-      <c r="C4">
-        <v>2.1269999999999998</v>
-      </c>
       <c r="D4">
+        <v>0.67300000000000004</v>
+      </c>
+      <c r="E4">
         <v>0.624</v>
       </c>
-      <c r="E4">
-        <v>0.67300000000000004</v>
-      </c>
       <c r="F4">
-        <f t="shared" si="0"/>
+        <f>AVERAGE(B4:C4)</f>
         <v>1.577</v>
       </c>
       <c r="G4">
         <v>4.2</v>
+      </c>
+      <c r="H4">
+        <f t="shared" si="0"/>
+        <v>2.1</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.4">

</xml_diff>